<commit_message>
print2xls2.py prints 3 different sheets to excel for each year. not finished yet but working.
</commit_message>
<xml_diff>
--- a/OECD_salaries/EIA_matrices.xlsx
+++ b/OECD_salaries/EIA_matrices.xlsx
@@ -37343,7 +37343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:AT20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37361,17 +37361,227 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Direct output impact</t>
+          <t>A01_02</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>Indirect output impact</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>Induced output impact</t>
+          <t>B05_06</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>B07_08</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>B09</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>C10T12</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>C13T15</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>C17_18</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="M2" s="14" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="N2" s="14" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="O2" s="14" t="inlineStr">
+        <is>
+          <t>C23</t>
+        </is>
+      </c>
+      <c r="P2" s="14" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="Q2" s="14" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="R2" s="14" t="inlineStr">
+        <is>
+          <t>C26</t>
+        </is>
+      </c>
+      <c r="S2" s="14" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="T2" s="14" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="U2" s="14" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="V2" s="14" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+      <c r="W2" s="14" t="inlineStr">
+        <is>
+          <t>C31T33</t>
+        </is>
+      </c>
+      <c r="X2" s="14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Y2" s="14" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Z2" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AA2" s="14" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AB2" s="14" t="inlineStr">
+        <is>
+          <t>H49</t>
+        </is>
+      </c>
+      <c r="AC2" s="14" t="inlineStr">
+        <is>
+          <t>H50</t>
+        </is>
+      </c>
+      <c r="AD2" s="14" t="inlineStr">
+        <is>
+          <t>H51</t>
+        </is>
+      </c>
+      <c r="AE2" s="14" t="inlineStr">
+        <is>
+          <t>H52</t>
+        </is>
+      </c>
+      <c r="AF2" s="14" t="inlineStr">
+        <is>
+          <t>H53</t>
+        </is>
+      </c>
+      <c r="AG2" s="14" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="AH2" s="14" t="inlineStr">
+        <is>
+          <t>J58T60</t>
+        </is>
+      </c>
+      <c r="AI2" s="14" t="inlineStr">
+        <is>
+          <t>J61</t>
+        </is>
+      </c>
+      <c r="AJ2" s="14" t="inlineStr">
+        <is>
+          <t>J62_63</t>
+        </is>
+      </c>
+      <c r="AK2" s="14" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="AL2" s="14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AM2" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AN2" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO2" s="14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="AP2" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AQ2" s="14" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AR2" s="14" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="AS2" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AT2" s="14" t="inlineStr">
+        <is>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -37382,13 +37592,139 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1757825.3</v>
+        <v>30566.3</v>
       </c>
       <c r="C3" t="n">
-        <v/>
+        <v>1721.7</v>
       </c>
       <c r="D3" t="n">
-        <v/>
+        <v>54701.2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13061</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3917.9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>61878.69999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3638.8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>9252.4</v>
+      </c>
+      <c r="J3" t="n">
+        <v>16189.4</v>
+      </c>
+      <c r="K3" t="n">
+        <v>20092.1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>17046.6</v>
+      </c>
+      <c r="M3" t="n">
+        <v>7182.700000000001</v>
+      </c>
+      <c r="N3" t="n">
+        <v>9342.4</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3482.3</v>
+      </c>
+      <c r="P3" t="n">
+        <v>33041.4</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>9157.5</v>
+      </c>
+      <c r="R3" t="n">
+        <v>8136.299999999999</v>
+      </c>
+      <c r="S3" t="n">
+        <v>4712.3</v>
+      </c>
+      <c r="T3" t="n">
+        <v>19292.2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>62711.5</v>
+      </c>
+      <c r="V3" t="n">
+        <v>18732.3</v>
+      </c>
+      <c r="W3" t="n">
+        <v>13428.6</v>
+      </c>
+      <c r="X3" t="n">
+        <v>23484</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>3871.8</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>221092.2</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>154197.8</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>29042.9</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>3643.7</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>12485.2</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>7618.1</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>2617.6</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>54483.9</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>15123.6</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>26066.7</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>17966.2</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>83458.7</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>197093.3</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>22504.1</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>17301.4</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>170410.7</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>96871.79999999999</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>134186.6</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>18412.8</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>22043.2</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>2563.4</v>
       </c>
     </row>
     <row r="4">
@@ -37398,13 +37734,139 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v/>
+        <v>38226.32438474995</v>
       </c>
       <c r="C4" t="n">
-        <v>994324.4450378901</v>
+        <v>1651.79469898397</v>
       </c>
       <c r="D4" t="n">
-        <v/>
+        <v>27536.10117972063</v>
+      </c>
+      <c r="E4" t="n">
+        <v>15630.95265239129</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15775.19924542876</v>
+      </c>
+      <c r="G4" t="n">
+        <v>26134.90509407771</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1559.188476602607</v>
+      </c>
+      <c r="I4" t="n">
+        <v>13459.97290124833</v>
+      </c>
+      <c r="J4" t="n">
+        <v>12780.80074849717</v>
+      </c>
+      <c r="K4" t="n">
+        <v>24065.21135663751</v>
+      </c>
+      <c r="L4" t="n">
+        <v>18044.74434594855</v>
+      </c>
+      <c r="M4" t="n">
+        <v>3103.294527374329</v>
+      </c>
+      <c r="N4" t="n">
+        <v>13803.76447996818</v>
+      </c>
+      <c r="O4" t="n">
+        <v>13154.86538194447</v>
+      </c>
+      <c r="P4" t="n">
+        <v>21072.42769713492</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>19873.08802793197</v>
+      </c>
+      <c r="R4" t="n">
+        <v>3360.500509383411</v>
+      </c>
+      <c r="S4" t="n">
+        <v>3584.694870647409</v>
+      </c>
+      <c r="T4" t="n">
+        <v>9193.489334365471</v>
+      </c>
+      <c r="U4" t="n">
+        <v>14445.24419154789</v>
+      </c>
+      <c r="V4" t="n">
+        <v>8227.328646391205</v>
+      </c>
+      <c r="W4" t="n">
+        <v>14891.18829951928</v>
+      </c>
+      <c r="X4" t="n">
+        <v>19477.99011708359</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>9249.396045247551</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>39533.33715883706</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>101512.1079209897</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>44887.41566285412</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>988.9991407215244</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>5301.095572974235</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>22305.1974025913</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>8434.19065368705</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>13193.39157884356</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>14903.25027949116</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>19145.88760183097</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>25689.67101896309</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>113500.2496495792</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>35525.08337637199</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>79789.47236360279</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>60283.06190341854</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>17311.38829026483</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>4566.196250296258</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>25726.99169003616</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>4029.495920295988</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>9395.494389414536</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -37414,13 +37876,139 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v/>
+        <v>41541.86515700947</v>
       </c>
       <c r="C5" t="n">
-        <v/>
+        <v>2317.732680844619</v>
       </c>
       <c r="D5" t="n">
-        <v>1492873.385581218</v>
+        <v>18413.40255960759</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3764.068808280145</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2780.22961902417</v>
+      </c>
+      <c r="G5" t="n">
+        <v>87322.51518309575</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4721.643208030258</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4146.094862980484</v>
+      </c>
+      <c r="J5" t="n">
+        <v>11639.77562619039</v>
+      </c>
+      <c r="K5" t="n">
+        <v>25702.05938662175</v>
+      </c>
+      <c r="L5" t="n">
+        <v>12758.4075494203</v>
+      </c>
+      <c r="M5" t="n">
+        <v>4179.908501142321</v>
+      </c>
+      <c r="N5" t="n">
+        <v>8178.464219433832</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4978.053630003916</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5683.532577877505</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>8589.036258863276</v>
+      </c>
+      <c r="R5" t="n">
+        <v>3802.120605486368</v>
+      </c>
+      <c r="S5" t="n">
+        <v>3610.901481420923</v>
+      </c>
+      <c r="T5" t="n">
+        <v>5420.623971674411</v>
+      </c>
+      <c r="U5" t="n">
+        <v>26851.72954765885</v>
+      </c>
+      <c r="V5" t="n">
+        <v>6808.701941264619</v>
+      </c>
+      <c r="W5" t="n">
+        <v>20131.67069571299</v>
+      </c>
+      <c r="X5" t="n">
+        <v>39646.89792625459</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>9770.533350331771</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>30637.03335024794</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>158994.2614394097</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>35175.7916383478</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1302.966808944178</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>5751.831749010964</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>15062.98564856123</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>7615.346724581292</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>77455.97201309858</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>25085.34989431465</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>48324.85258667594</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>17470.72212084875</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>183768.4183257671</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>289752.5828704715</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>48663.03133776773</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>44315.64107783175</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>22101.46121264019</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>18623.44821422076</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>50833.92186065586</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>26107.82490570346</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>19322.87729435618</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>3747.095159531646</v>
       </c>
     </row>
     <row r="6">
@@ -37430,13 +38018,139 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v/>
+        <v>110334.4895417594</v>
       </c>
       <c r="C6" t="n">
-        <v/>
+        <v>5691.22737982859</v>
       </c>
       <c r="D6" t="n">
-        <v/>
+        <v>100650.7037393282</v>
+      </c>
+      <c r="E6" t="n">
+        <v>32456.02146067143</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22473.32886445292</v>
+      </c>
+      <c r="G6" t="n">
+        <v>175336.1202771734</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9919.631684632865</v>
+      </c>
+      <c r="I6" t="n">
+        <v>26858.46776422882</v>
+      </c>
+      <c r="J6" t="n">
+        <v>40609.97637468755</v>
+      </c>
+      <c r="K6" t="n">
+        <v>69859.37074325926</v>
+      </c>
+      <c r="L6" t="n">
+        <v>47849.75189536886</v>
+      </c>
+      <c r="M6" t="n">
+        <v>14465.90302851665</v>
+      </c>
+      <c r="N6" t="n">
+        <v>31324.62869940202</v>
+      </c>
+      <c r="O6" t="n">
+        <v>21615.21901194838</v>
+      </c>
+      <c r="P6" t="n">
+        <v>59797.36027501243</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>37619.62428679525</v>
+      </c>
+      <c r="R6" t="n">
+        <v>15298.92111486978</v>
+      </c>
+      <c r="S6" t="n">
+        <v>11907.89635206833</v>
+      </c>
+      <c r="T6" t="n">
+        <v>33906.31330603988</v>
+      </c>
+      <c r="U6" t="n">
+        <v>104008.4737392067</v>
+      </c>
+      <c r="V6" t="n">
+        <v>33768.33058765582</v>
+      </c>
+      <c r="W6" t="n">
+        <v>48451.45899523226</v>
+      </c>
+      <c r="X6" t="n">
+        <v>82608.8880433382</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>22891.72939557932</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>291262.570509085</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>414704.1693603994</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>109106.1073012019</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>5935.665949665703</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>23538.1273219852</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>44986.28305115253</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>18667.13737826834</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>145133.2635919421</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>55112.20017380582</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>93537.44018850691</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>61126.59313981185</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>380727.3679753464</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>522370.9662468435</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>150956.6037013705</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>121900.1029812503</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>209823.549502905</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>120061.444464517</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>210747.513550692</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>48550.12082599945</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>50761.57168377072</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>6310.495159531647</v>
       </c>
     </row>
     <row r="8">
@@ -37454,17 +38168,227 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Direct income impact</t>
+          <t>A01_02</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>Indirect income impact</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>Induced income impact</t>
+          <t>B05_06</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>B07_08</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>B09</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>C10T12</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>C13T15</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>C17_18</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="M9" s="14" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="N9" s="14" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>C23</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="Q9" s="14" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="R9" s="14" t="inlineStr">
+        <is>
+          <t>C26</t>
+        </is>
+      </c>
+      <c r="S9" s="14" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="T9" s="14" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="U9" s="14" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="V9" s="14" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+      <c r="W9" s="14" t="inlineStr">
+        <is>
+          <t>C31T33</t>
+        </is>
+      </c>
+      <c r="X9" s="14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Y9" s="14" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Z9" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AA9" s="14" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AB9" s="14" t="inlineStr">
+        <is>
+          <t>H49</t>
+        </is>
+      </c>
+      <c r="AC9" s="14" t="inlineStr">
+        <is>
+          <t>H50</t>
+        </is>
+      </c>
+      <c r="AD9" s="14" t="inlineStr">
+        <is>
+          <t>H51</t>
+        </is>
+      </c>
+      <c r="AE9" s="14" t="inlineStr">
+        <is>
+          <t>H52</t>
+        </is>
+      </c>
+      <c r="AF9" s="14" t="inlineStr">
+        <is>
+          <t>H53</t>
+        </is>
+      </c>
+      <c r="AG9" s="14" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="AH9" s="14" t="inlineStr">
+        <is>
+          <t>J58T60</t>
+        </is>
+      </c>
+      <c r="AI9" s="14" t="inlineStr">
+        <is>
+          <t>J61</t>
+        </is>
+      </c>
+      <c r="AJ9" s="14" t="inlineStr">
+        <is>
+          <t>J62_63</t>
+        </is>
+      </c>
+      <c r="AK9" s="14" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="AL9" s="14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AM9" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AN9" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO9" s="14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="AP9" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AQ9" s="14" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AR9" s="14" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="AS9" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AT9" s="14" t="inlineStr">
+        <is>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -37475,13 +38399,139 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>516981.3226262787</v>
+        <v>3198.357093163043</v>
       </c>
       <c r="C10" t="n">
-        <v/>
+        <v>209.1269962653388</v>
       </c>
       <c r="D10" t="n">
-        <v/>
+        <v>8111.794456286868</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2468.671026767043</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1535.539227952938</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9064.310618574153</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1021.456842753261</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2006.607401145615</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3634.539859164653</v>
+      </c>
+      <c r="K10" t="n">
+        <v>502.0636170935526</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2052.074228654965</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1580.862963611087</v>
+      </c>
+      <c r="N10" t="n">
+        <v>2216.30092583392</v>
+      </c>
+      <c r="O10" t="n">
+        <v>735.876419392453</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3154.179401263998</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>2901.109425162242</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2363.67204241217</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1144.964180687461</v>
+      </c>
+      <c r="T10" t="n">
+        <v>5712.389686089209</v>
+      </c>
+      <c r="U10" t="n">
+        <v>7223.456692510277</v>
+      </c>
+      <c r="V10" t="n">
+        <v>4474.520661068124</v>
+      </c>
+      <c r="W10" t="n">
+        <v>2685.34066101695</v>
+      </c>
+      <c r="X10" t="n">
+        <v>5565.026577098725</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>648.6491803278689</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>63300.49473378468</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>64246.10844323648</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>7495.978531912535</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>716.532983637698</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>2610.153189814633</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>2146.372879390436</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>1087.194896805074</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>19709.88015355268</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>4671.175329035008</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>7168.561579710511</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>26409.23135762704</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>8066.124703000581</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>8734.200124054923</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>6739.412748888956</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>77310.64849591577</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>60015.92005197268</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>64897.36517980032</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>5712.085039791108</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>9169.592020051658</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>2563.4</v>
       </c>
     </row>
     <row r="11">
@@ -37491,13 +38541,139 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v/>
+        <v>3999.876849390223</v>
       </c>
       <c r="C11" t="n">
-        <v>278653.514507568</v>
+        <v>200.635920221599</v>
       </c>
       <c r="D11" t="n">
-        <v/>
+        <v>4083.405718657217</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2954.420024020048</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6182.760476308595</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3828.375479117634</v>
+      </c>
+      <c r="H11" t="n">
+        <v>437.6837799735532</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2919.121659554743</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2869.305209115495</v>
+      </c>
+      <c r="K11" t="n">
+        <v>601.3441631205433</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2172.231109722081</v>
+      </c>
+      <c r="M11" t="n">
+        <v>683.0138225880308</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3274.672032555539</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2779.874001336768</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2011.604150457545</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>6295.82342177585</v>
+      </c>
+      <c r="R11" t="n">
+        <v>976.2571565135783</v>
+      </c>
+      <c r="S11" t="n">
+        <v>870.9859783089687</v>
+      </c>
+      <c r="T11" t="n">
+        <v>2722.177545992706</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1663.882953371898</v>
+      </c>
+      <c r="V11" t="n">
+        <v>1965.233954916112</v>
+      </c>
+      <c r="W11" t="n">
+        <v>2977.817004867145</v>
+      </c>
+      <c r="X11" t="n">
+        <v>4615.718475133558</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>1549.566910294348</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>11318.71590509253</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>42294.75319228565</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>11585.45132069418</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>194.4865123682832</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>1108.245884672326</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>6284.410912743593</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>3503.059687259174</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>4772.78915125198</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>4603.116653970827</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>10250.24705624681</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>35915.42106627786</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>1453.878709211878</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>30967.56677300831</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>23482.0555523808</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>7853.700824449263</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>2828.939578901159</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>12442.47916473005</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>1250.044716948102</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>3908.36404776147</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -37507,13 +38683,139 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v/>
+        <v>4346.804130305072</v>
       </c>
       <c r="C12" t="n">
-        <v/>
+        <v>281.5243501719499</v>
       </c>
       <c r="D12" t="n">
-        <v>367399.09490271</v>
+        <v>2730.575139199931</v>
+      </c>
+      <c r="E12" t="n">
+        <v>711.4499356679235</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1089.653039313986</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12791.45168878366</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1325.424525635364</v>
+      </c>
+      <c r="I12" t="n">
+        <v>899.1812543673479</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2613.143690632277</v>
+      </c>
+      <c r="K12" t="n">
+        <v>642.2459027379225</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1535.860484251542</v>
+      </c>
+      <c r="M12" t="n">
+        <v>919.9691676861107</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1940.18002027646</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1051.95769485423</v>
+      </c>
+      <c r="P12" t="n">
+        <v>542.5581659237832</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>2721.019278585693</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1104.551967978978</v>
+      </c>
+      <c r="S12" t="n">
+        <v>877.3534911228585</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1605.038122555272</v>
+      </c>
+      <c r="U12" t="n">
+        <v>3092.930411591372</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1626.371428561532</v>
+      </c>
+      <c r="W12" t="n">
+        <v>4025.765447880006</v>
+      </c>
+      <c r="X12" t="n">
+        <v>9395.164395295826</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>1636.873921447081</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>8771.631781881748</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>66244.54150635489</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>9078.879139620476</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>256.2282007831769</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>1202.476691359213</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>4243.943224520442</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>3162.960764198509</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>28020.16605924141</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>7748.027423796818</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>6970.864588244309</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>58150.71018108803</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>11858.24412321339</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>18886.89858057952</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>17262.26758846836</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>10026.82518795206</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>11537.96439331907</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>24585.07474302515</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>8099.263342096499</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>8037.984568609174</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>3747.095159531646</v>
       </c>
     </row>
     <row r="13">
@@ -37523,13 +38825,139 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v/>
+        <v>110334.4895417594</v>
       </c>
       <c r="C13" t="n">
-        <v/>
+        <v>5691.22737982859</v>
       </c>
       <c r="D13" t="n">
-        <v/>
+        <v>100650.7037393282</v>
+      </c>
+      <c r="E13" t="n">
+        <v>32456.02146067143</v>
+      </c>
+      <c r="F13" t="n">
+        <v>22473.32886445292</v>
+      </c>
+      <c r="G13" t="n">
+        <v>175336.1202771734</v>
+      </c>
+      <c r="H13" t="n">
+        <v>9919.631684632865</v>
+      </c>
+      <c r="I13" t="n">
+        <v>26858.46776422882</v>
+      </c>
+      <c r="J13" t="n">
+        <v>40609.97637468755</v>
+      </c>
+      <c r="K13" t="n">
+        <v>69859.37074325926</v>
+      </c>
+      <c r="L13" t="n">
+        <v>47849.75189536886</v>
+      </c>
+      <c r="M13" t="n">
+        <v>14465.90302851665</v>
+      </c>
+      <c r="N13" t="n">
+        <v>31324.62869940202</v>
+      </c>
+      <c r="O13" t="n">
+        <v>21615.21901194838</v>
+      </c>
+      <c r="P13" t="n">
+        <v>59797.36027501243</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>37619.62428679525</v>
+      </c>
+      <c r="R13" t="n">
+        <v>15298.92111486978</v>
+      </c>
+      <c r="S13" t="n">
+        <v>11907.89635206833</v>
+      </c>
+      <c r="T13" t="n">
+        <v>33906.31330603988</v>
+      </c>
+      <c r="U13" t="n">
+        <v>104008.4737392067</v>
+      </c>
+      <c r="V13" t="n">
+        <v>33768.33058765582</v>
+      </c>
+      <c r="W13" t="n">
+        <v>48451.45899523226</v>
+      </c>
+      <c r="X13" t="n">
+        <v>82608.8880433382</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>22891.72939557932</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>291262.570509085</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>414704.1693603994</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>109106.1073012019</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>5935.665949665703</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>23538.1273219852</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>44986.28305115253</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>18667.13737826834</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>145133.2635919421</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>55112.20017380582</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>93537.44018850691</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>61126.59313981185</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>380727.3679753464</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>522370.9662468435</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>150956.6037013705</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>121900.1029812503</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>209823.549502905</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>120061.444464517</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>210747.513550692</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>48550.12082599945</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>50761.57168377072</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>6310.495159531647</v>
       </c>
     </row>
     <row r="15">
@@ -37547,17 +38975,227 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Direct GDP impact</t>
+          <t>A01_02</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Indirect GDP impact</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Induced GDP impact</t>
+          <t>B05_06</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>B07_08</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>B09</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>C10T12</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>C13T15</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>C17_18</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="M16" s="14" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="N16" s="14" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="O16" s="14" t="inlineStr">
+        <is>
+          <t>C23</t>
+        </is>
+      </c>
+      <c r="P16" s="14" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="Q16" s="14" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="R16" s="14" t="inlineStr">
+        <is>
+          <t>C26</t>
+        </is>
+      </c>
+      <c r="S16" s="14" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="T16" s="14" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="U16" s="14" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="V16" s="14" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+      <c r="W16" s="14" t="inlineStr">
+        <is>
+          <t>C31T33</t>
+        </is>
+      </c>
+      <c r="X16" s="14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Y16" s="14" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Z16" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AA16" s="14" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AB16" s="14" t="inlineStr">
+        <is>
+          <t>H49</t>
+        </is>
+      </c>
+      <c r="AC16" s="14" t="inlineStr">
+        <is>
+          <t>H50</t>
+        </is>
+      </c>
+      <c r="AD16" s="14" t="inlineStr">
+        <is>
+          <t>H51</t>
+        </is>
+      </c>
+      <c r="AE16" s="14" t="inlineStr">
+        <is>
+          <t>H52</t>
+        </is>
+      </c>
+      <c r="AF16" s="14" t="inlineStr">
+        <is>
+          <t>H53</t>
+        </is>
+      </c>
+      <c r="AG16" s="14" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="AH16" s="14" t="inlineStr">
+        <is>
+          <t>J58T60</t>
+        </is>
+      </c>
+      <c r="AI16" s="14" t="inlineStr">
+        <is>
+          <t>J61</t>
+        </is>
+      </c>
+      <c r="AJ16" s="14" t="inlineStr">
+        <is>
+          <t>J62_63</t>
+        </is>
+      </c>
+      <c r="AK16" s="14" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="AL16" s="14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AM16" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AN16" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO16" s="14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="AP16" s="14" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AQ16" s="14" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AR16" s="14" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="AS16" s="14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AT16" s="14" t="inlineStr">
+        <is>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -37568,13 +39206,139 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>942368.4176838958</v>
+        <v>12157.81810595081</v>
       </c>
       <c r="C17" t="n">
-        <v/>
+        <v>890.0400053352301</v>
       </c>
       <c r="D17" t="n">
-        <v/>
+        <v>26569.93157606098</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7921.360846228914</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2351.026484910959</v>
+      </c>
+      <c r="G17" t="n">
+        <v>16797.94413244756</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1342.972144203763</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2854.948769631088</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5617.447971694857</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4868.524636410988</v>
+      </c>
+      <c r="L17" t="n">
+        <v>5600.394896170845</v>
+      </c>
+      <c r="M17" t="n">
+        <v>2789.606189906768</v>
+      </c>
+      <c r="N17" t="n">
+        <v>3232.08365425741</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1194.653233678339</v>
+      </c>
+      <c r="P17" t="n">
+        <v>5419.036277857856</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>3785.889443280929</v>
+      </c>
+      <c r="R17" t="n">
+        <v>3485.883712717562</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1643.443873836957</v>
+      </c>
+      <c r="T17" t="n">
+        <v>7865.659760301624</v>
+      </c>
+      <c r="U17" t="n">
+        <v>11862.1784680208</v>
+      </c>
+      <c r="V17" t="n">
+        <v>7264.416985170293</v>
+      </c>
+      <c r="W17" t="n">
+        <v>5863.0633220339</v>
+      </c>
+      <c r="X17" t="n">
+        <v>17100.29294861947</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>2235.334426229508</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>99055.56276235441</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>93317.25708552658</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>14397.70471728739</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>1147.239308379743</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>4893.124688102641</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>3816.764080473215</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>1417.974234294556</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>25980.14444590563</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>7175.036917195076</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>14795.821123094</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>10548.28677000465</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>45651.34630545123</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>149208.1406575923</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>14156.52017930776</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>10691.88467302874</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>94149.44666991971</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>77039.21849624252</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>90919.89975768149</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>8994.886875618255</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>11734.80607147856</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>2563.4</v>
       </c>
     </row>
     <row r="18">
@@ -37584,13 +39348,139 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v/>
+        <v>15204.61091885056</v>
       </c>
       <c r="C18" t="n">
-        <v>509813.6082791861</v>
+        <v>853.9021680295042</v>
       </c>
       <c r="D18" t="n">
-        <v/>
+        <v>13375.06899696294</v>
+      </c>
+      <c r="E18" t="n">
+        <v>9480.010437938163</v>
+      </c>
+      <c r="F18" t="n">
+        <v>9466.273062291119</v>
+      </c>
+      <c r="G18" t="n">
+        <v>7094.730103850544</v>
+      </c>
+      <c r="H18" t="n">
+        <v>575.4497888426959</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4153.250299780239</v>
+      </c>
+      <c r="J18" t="n">
+        <v>4434.721684638191</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5831.250808538042</v>
+      </c>
+      <c r="L18" t="n">
+        <v>5928.319672999778</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1205.252846793995</v>
+      </c>
+      <c r="N18" t="n">
+        <v>4775.531077980412</v>
+      </c>
+      <c r="O18" t="n">
+        <v>4512.966277214254</v>
+      </c>
+      <c r="P18" t="n">
+        <v>3456.035463185906</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>8215.922923324082</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1439.759349119219</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1250.184586028107</v>
+      </c>
+      <c r="T18" t="n">
+        <v>3748.295120000864</v>
+      </c>
+      <c r="U18" t="n">
+        <v>2732.386637447389</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3190.571684279153</v>
+      </c>
+      <c r="W18" t="n">
+        <v>6501.644247383331</v>
+      </c>
+      <c r="X18" t="n">
+        <v>14183.24548852173</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>5340.021024271119</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>17712.05388585623</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>61432.98719019796</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>22252.4526213262</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>311.3919066304916</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>2077.573576883978</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>11175.184921972</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>4568.866531959121</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>6291.146906696304</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>7070.497166120958</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>10867.47183953298</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>15082.87879101314</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>62083.87145388209</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>26894.02246192238</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>50192.68824843746</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>37253.60639072002</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>9564.291612067547</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>3631.358048712804</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>17431.66236811121</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>1968.459982665738</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>5001.737706206196</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -37600,13 +39490,139 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v/>
+        <v>16523.37510136513</v>
       </c>
       <c r="C19" t="n">
-        <v/>
+        <v>1198.161588908975</v>
       </c>
       <c r="D19" t="n">
-        <v>832932.8289969413</v>
+        <v>8943.914321646324</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2282.868637962015</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1668.341067525901</v>
+      </c>
+      <c r="G19" t="n">
+        <v>23705.06703519056</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1742.617154900937</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1279.331679114598</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4038.805266552586</v>
+      </c>
+      <c r="K19" t="n">
+        <v>6227.876097086233</v>
+      </c>
+      <c r="L19" t="n">
+        <v>4191.576063440276</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1623.386557705395</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2829.410057432905</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1707.793086898995</v>
+      </c>
+      <c r="P19" t="n">
+        <v>932.1417744376802</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>3550.875424557751</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1628.965290421047</v>
+      </c>
+      <c r="S19" t="n">
+        <v>1259.324304197527</v>
+      </c>
+      <c r="T19" t="n">
+        <v>2210.052966987993</v>
+      </c>
+      <c r="U19" t="n">
+        <v>5079.132345253371</v>
+      </c>
+      <c r="V19" t="n">
+        <v>2640.425896931218</v>
+      </c>
+      <c r="W19" t="n">
+        <v>8789.692154602822</v>
+      </c>
+      <c r="X19" t="n">
+        <v>28869.59500268129</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>5640.893011162803</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>13726.25800402651</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>96219.97440861558</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>17438.01966076935</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>410.2463816271591</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>2254.223395131688</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>7546.745588547278</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>4125.292420796039</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>36934.16479177013</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>11901.15525221926</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>27429.85781369885</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>10257.38258562058</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>100520.0860424932</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>219355.2197910227</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>30612.16334443034</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>27386.09150794225</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>12210.73761076486</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>14810.66622204615</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>34443.19387972156</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>12754.00436626974</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>10286.62888293197</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>3747.095159531646</v>
       </c>
     </row>
     <row r="20">
@@ -37616,20 +39632,146 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v/>
+        <v>110334.4895417594</v>
       </c>
       <c r="C20" t="n">
-        <v/>
+        <v>5691.22737982859</v>
       </c>
       <c r="D20" t="n">
-        <v/>
+        <v>100650.7037393282</v>
+      </c>
+      <c r="E20" t="n">
+        <v>32456.02146067143</v>
+      </c>
+      <c r="F20" t="n">
+        <v>22473.32886445292</v>
+      </c>
+      <c r="G20" t="n">
+        <v>175336.1202771734</v>
+      </c>
+      <c r="H20" t="n">
+        <v>9919.631684632865</v>
+      </c>
+      <c r="I20" t="n">
+        <v>26858.46776422882</v>
+      </c>
+      <c r="J20" t="n">
+        <v>40609.97637468755</v>
+      </c>
+      <c r="K20" t="n">
+        <v>69859.37074325926</v>
+      </c>
+      <c r="L20" t="n">
+        <v>47849.75189536886</v>
+      </c>
+      <c r="M20" t="n">
+        <v>14465.90302851665</v>
+      </c>
+      <c r="N20" t="n">
+        <v>31324.62869940202</v>
+      </c>
+      <c r="O20" t="n">
+        <v>21615.21901194838</v>
+      </c>
+      <c r="P20" t="n">
+        <v>59797.36027501243</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>37619.62428679525</v>
+      </c>
+      <c r="R20" t="n">
+        <v>15298.92111486978</v>
+      </c>
+      <c r="S20" t="n">
+        <v>11907.89635206833</v>
+      </c>
+      <c r="T20" t="n">
+        <v>33906.31330603988</v>
+      </c>
+      <c r="U20" t="n">
+        <v>104008.4737392067</v>
+      </c>
+      <c r="V20" t="n">
+        <v>33768.33058765582</v>
+      </c>
+      <c r="W20" t="n">
+        <v>48451.45899523226</v>
+      </c>
+      <c r="X20" t="n">
+        <v>82608.8880433382</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>22891.72939557932</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>291262.570509085</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>414704.1693603994</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>109106.1073012019</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>5935.665949665703</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>23538.1273219852</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>44986.28305115253</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>18667.13737826834</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>145133.2635919421</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>55112.20017380582</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>93537.44018850691</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>61126.59313981185</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>380727.3679753464</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>522370.9662468435</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>150956.6037013705</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>121900.1029812503</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>209823.549502905</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>120061.444464517</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>210747.513550692</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>48550.12082599945</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>50761.57168377072</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>6310.495159531647</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A8:AT8"/>
+    <mergeCell ref="A15:AT15"/>
+    <mergeCell ref="A1:AT1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
func_data_upload_OECD_salaries3.py updated to read and output TTL as well as DOM tables
</commit_message>
<xml_diff>
--- a/OECD_salaries/EIA_matrices.xlsx
+++ b/OECD_salaries/EIA_matrices.xlsx
@@ -39246,136 +39246,136 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>110334.4895417594</v>
+        <v>11545.03807285834</v>
       </c>
       <c r="C13" t="n">
-        <v>5691.22737982859</v>
+        <v>691.2872666588878</v>
       </c>
       <c r="D13" t="n">
-        <v>100650.7037393282</v>
+        <v>14925.77531414402</v>
       </c>
       <c r="E13" t="n">
-        <v>32456.02146067143</v>
+        <v>6134.540986455015</v>
       </c>
       <c r="F13" t="n">
-        <v>22473.32886445292</v>
+        <v>8807.952743575517</v>
       </c>
       <c r="G13" t="n">
-        <v>175336.1202771734</v>
+        <v>25684.13778647545</v>
       </c>
       <c r="H13" t="n">
-        <v>9919.631684632865</v>
+        <v>2784.565148362179</v>
       </c>
       <c r="I13" t="n">
-        <v>26858.46776422882</v>
+        <v>5824.910315067706</v>
       </c>
       <c r="J13" t="n">
-        <v>40609.97637468755</v>
+        <v>9116.988758912425</v>
       </c>
       <c r="K13" t="n">
-        <v>69859.37074325926</v>
+        <v>1745.653682952018</v>
       </c>
       <c r="L13" t="n">
-        <v>47849.75189536886</v>
+        <v>5760.165822628589</v>
       </c>
       <c r="M13" t="n">
-        <v>14465.90302851665</v>
+        <v>3183.845953885228</v>
       </c>
       <c r="N13" t="n">
-        <v>31324.62869940202</v>
+        <v>7431.152978665918</v>
       </c>
       <c r="O13" t="n">
-        <v>21615.21901194838</v>
+        <v>4567.708115583451</v>
       </c>
       <c r="P13" t="n">
-        <v>59797.36027501243</v>
+        <v>5708.341717645328</v>
       </c>
       <c r="Q13" t="n">
-        <v>37619.62428679525</v>
+        <v>11917.95212552379</v>
       </c>
       <c r="R13" t="n">
-        <v>15298.92111486978</v>
+        <v>4444.481166904726</v>
       </c>
       <c r="S13" t="n">
-        <v>11907.89635206833</v>
+        <v>2893.303650119288</v>
       </c>
       <c r="T13" t="n">
-        <v>33906.31330603988</v>
+        <v>10039.60535463719</v>
       </c>
       <c r="U13" t="n">
-        <v>104008.4737392067</v>
+        <v>11980.27005747355</v>
       </c>
       <c r="V13" t="n">
-        <v>33768.33058765582</v>
+        <v>8066.126044545769</v>
       </c>
       <c r="W13" t="n">
-        <v>48451.45899523226</v>
+        <v>9688.9231137641</v>
       </c>
       <c r="X13" t="n">
-        <v>82608.8880433382</v>
+        <v>19575.90944752811</v>
       </c>
       <c r="Y13" t="n">
-        <v>22891.72939557932</v>
+        <v>3835.090012069297</v>
       </c>
       <c r="Z13" t="n">
-        <v>291262.570509085</v>
+        <v>83390.84242075897</v>
       </c>
       <c r="AA13" t="n">
-        <v>414704.1693603994</v>
+        <v>172785.403141877</v>
       </c>
       <c r="AB13" t="n">
-        <v>109106.1073012019</v>
+        <v>28160.30899222719</v>
       </c>
       <c r="AC13" t="n">
-        <v>5935.665949665703</v>
+        <v>1167.247696789158</v>
       </c>
       <c r="AD13" t="n">
-        <v>23538.1273219852</v>
+        <v>4920.875765846173</v>
       </c>
       <c r="AE13" t="n">
-        <v>44986.28305115253</v>
+        <v>12674.72701665447</v>
       </c>
       <c r="AF13" t="n">
-        <v>18667.13737826834</v>
+        <v>7753.215348262758</v>
       </c>
       <c r="AG13" t="n">
-        <v>145133.2635919421</v>
+        <v>52502.83536404606</v>
       </c>
       <c r="AH13" t="n">
-        <v>55112.20017380582</v>
+        <v>17022.31940680265</v>
       </c>
       <c r="AI13" t="n">
-        <v>93537.44018850691</v>
+        <v>0</v>
       </c>
       <c r="AJ13" t="n">
-        <v>61126.59313981185</v>
+        <v>24389.67322420163</v>
       </c>
       <c r="AK13" t="n">
-        <v>380727.3679753464</v>
+        <v>120475.3626049929</v>
       </c>
       <c r="AL13" t="n">
-        <v>522370.9662468435</v>
+        <v>21378.24753542585</v>
       </c>
       <c r="AM13" t="n">
-        <v>150956.6037013705</v>
+        <v>58588.66547764276</v>
       </c>
       <c r="AN13" t="n">
-        <v>121900.1029812503</v>
+        <v>47483.73588973811</v>
       </c>
       <c r="AO13" t="n">
-        <v>209823.549502905</v>
+        <v>95191.1745083171</v>
       </c>
       <c r="AP13" t="n">
-        <v>120061.444464517</v>
+        <v>74382.8240241929</v>
       </c>
       <c r="AQ13" t="n">
-        <v>210747.513550692</v>
+        <v>101924.9190875555</v>
       </c>
       <c r="AR13" t="n">
-        <v>48550.12082599945</v>
+        <v>15061.39309883571</v>
       </c>
       <c r="AS13" t="n">
-        <v>50761.57168377072</v>
+        <v>21115.9406364223</v>
       </c>
       <c r="AT13" t="n">
         <v>6310.495159531647</v>
@@ -40053,136 +40053,136 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>110334.4895417594</v>
+        <v>43885.8041261665</v>
       </c>
       <c r="C20" t="n">
-        <v>5691.22737982859</v>
+        <v>2942.103762273709</v>
       </c>
       <c r="D20" t="n">
-        <v>100650.7037393282</v>
+        <v>48888.91489467024</v>
       </c>
       <c r="E20" t="n">
-        <v>32456.02146067143</v>
+        <v>19684.23992212909</v>
       </c>
       <c r="F20" t="n">
-        <v>22473.32886445292</v>
+        <v>13485.64061472798</v>
       </c>
       <c r="G20" t="n">
-        <v>175336.1202771734</v>
+        <v>47597.74127148866</v>
       </c>
       <c r="H20" t="n">
-        <v>9919.631684632865</v>
+        <v>3661.039087947396</v>
       </c>
       <c r="I20" t="n">
-        <v>26858.46776422882</v>
+        <v>8287.530748525925</v>
       </c>
       <c r="J20" t="n">
-        <v>40609.97637468755</v>
+        <v>14090.97492288563</v>
       </c>
       <c r="K20" t="n">
-        <v>69859.37074325926</v>
+        <v>16927.65154203526</v>
       </c>
       <c r="L20" t="n">
-        <v>47849.75189536886</v>
+        <v>15720.2906326109</v>
       </c>
       <c r="M20" t="n">
-        <v>14465.90302851665</v>
+        <v>5618.245594406157</v>
       </c>
       <c r="N20" t="n">
-        <v>31324.62869940202</v>
+        <v>10837.02478967073</v>
       </c>
       <c r="O20" t="n">
-        <v>21615.21901194838</v>
+        <v>7415.412597791587</v>
       </c>
       <c r="P20" t="n">
-        <v>59797.36027501243</v>
+        <v>9807.213515481442</v>
       </c>
       <c r="Q20" t="n">
-        <v>37619.62428679525</v>
+        <v>15552.68779116276</v>
       </c>
       <c r="R20" t="n">
-        <v>15298.92111486978</v>
+        <v>6554.608352257828</v>
       </c>
       <c r="S20" t="n">
-        <v>11907.89635206833</v>
+        <v>4152.952764062591</v>
       </c>
       <c r="T20" t="n">
-        <v>33906.31330603988</v>
+        <v>13824.00784729048</v>
       </c>
       <c r="U20" t="n">
-        <v>104008.4737392067</v>
+        <v>19673.69745072156</v>
       </c>
       <c r="V20" t="n">
-        <v>33768.33058765582</v>
+        <v>13095.41456638066</v>
       </c>
       <c r="W20" t="n">
-        <v>48451.45899523226</v>
+        <v>21154.39972402005</v>
       </c>
       <c r="X20" t="n">
-        <v>82608.8880433382</v>
+        <v>60153.13343982248</v>
       </c>
       <c r="Y20" t="n">
-        <v>22891.72939557932</v>
+        <v>13216.24846166343</v>
       </c>
       <c r="Z20" t="n">
-        <v>291262.570509085</v>
+        <v>130493.8746522371</v>
       </c>
       <c r="AA20" t="n">
-        <v>414704.1693603994</v>
+        <v>250970.2186843401</v>
       </c>
       <c r="AB20" t="n">
-        <v>109106.1073012019</v>
+        <v>54088.17699938294</v>
       </c>
       <c r="AC20" t="n">
-        <v>5935.665949665703</v>
+        <v>1868.877596637394</v>
       </c>
       <c r="AD20" t="n">
-        <v>23538.1273219852</v>
+        <v>9224.921660118305</v>
       </c>
       <c r="AE20" t="n">
-        <v>44986.28305115253</v>
+        <v>22538.6945909925</v>
       </c>
       <c r="AF20" t="n">
-        <v>18667.13737826834</v>
+        <v>10112.13318704971</v>
       </c>
       <c r="AG20" t="n">
-        <v>145133.2635919421</v>
+        <v>69205.45614437206</v>
       </c>
       <c r="AH20" t="n">
-        <v>55112.20017380582</v>
+        <v>26146.6893355353</v>
       </c>
       <c r="AI20" t="n">
-        <v>93537.44018850691</v>
+        <v>53093.15077632583</v>
       </c>
       <c r="AJ20" t="n">
-        <v>61126.59313981185</v>
+        <v>35888.54814663838</v>
       </c>
       <c r="AK20" t="n">
-        <v>380727.3679753464</v>
+        <v>208255.3038018265</v>
       </c>
       <c r="AL20" t="n">
-        <v>522370.9662468435</v>
+        <v>395457.3829105374</v>
       </c>
       <c r="AM20" t="n">
-        <v>150956.6037013705</v>
+        <v>94961.37177217555</v>
       </c>
       <c r="AN20" t="n">
-        <v>121900.1029812503</v>
+        <v>75331.58257169099</v>
       </c>
       <c r="AO20" t="n">
-        <v>209823.549502905</v>
+        <v>115924.4758927521</v>
       </c>
       <c r="AP20" t="n">
-        <v>120061.444464517</v>
+        <v>95481.24276700149</v>
       </c>
       <c r="AQ20" t="n">
-        <v>210747.513550692</v>
+        <v>142794.7560055143</v>
       </c>
       <c r="AR20" t="n">
-        <v>48550.12082599945</v>
+        <v>23717.35122455373</v>
       </c>
       <c r="AS20" t="n">
-        <v>50761.57168377072</v>
+        <v>27023.17266061672</v>
       </c>
       <c r="AT20" t="n">
         <v>6310.495159531647</v>

</xml_diff>